<commit_message>
refactor: simplify lead generation data model by removing deprecated contact and location fields
</commit_message>
<xml_diff>
--- a/frontend/public/templates/sample_lead_generation_upload.xlsx
+++ b/frontend/public/templates/sample_lead_generation_upload.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Generation Template" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,9 +26,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="12"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -40,8 +45,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00f96331"/>
-        <bgColor rgb="00f96331"/>
+        <fgColor rgb="00F96331"/>
+        <bgColor rgb="00F96331"/>
       </patternFill>
     </fill>
   </fills>
@@ -55,16 +60,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00D9D9D9"/>
       </left>
       <right style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00D9D9D9"/>
       </right>
       <top style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00D9D9D9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00D9D9D9"/>
       </bottom>
     </border>
   </borders>
@@ -76,8 +81,8 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -444,24 +449,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
-    <col width="42" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="39" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Subject Code</t>
@@ -500,26 +501,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>LinkedIn URL</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Instructions</t>
         </is>
       </c>
     </row>
@@ -539,47 +520,27 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Tech Innovators 1 LLC</t>
+          <t>Calgon Carbon Corporation</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://innovators1.io</t>
+          <t>calgoncarbon.com</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Jane Smith 1</t>
+          <t>Doug Conley</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>CTO</t>
+          <t>Marketing Manager</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>jsmith1@innovators.io</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>https://linkedin.com/company/innovators1</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>123-456-7891</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>Silicon Valley, Zone 1</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Extract B2B lead information for the tech sector in region 1.</t>
+          <t>dconley@calgoncarbon.com</t>
         </is>
       </c>
     </row>
@@ -591,235 +552,35 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>FRESHER</t>
+          <t>EXPERIENCED</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Tech Innovators 2 LLC</t>
+          <t>American Tank &amp; Fabricating Company</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://innovators2.io</t>
+          <t>atfco.com</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Jane Smith 2</t>
+          <t>Ted Thorbjornsen</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>CTO</t>
+          <t>General Manager</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>jsmith2@innovators.io</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>https://linkedin.com/company/innovators2</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>123-456-7892</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Silicon Valley, Zone 2</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>Extract B2B lead information for the tech sector in region 2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>LEAD_GENERATION</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>FRESHER</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Tech Innovators 3 LLC</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://innovators3.io</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Jane Smith 3</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>CTO</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>jsmith3@innovators.io</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>https://linkedin.com/company/innovators3</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>123-456-7893</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>Silicon Valley, Zone 3</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>Extract B2B lead information for the tech sector in region 3.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>LEAD_GENERATION</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>FRESHER</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Tech Innovators 4 LLC</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>https://innovators4.io</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Jane Smith 4</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>CTO</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>jsmith4@innovators.io</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>https://linkedin.com/company/innovators4</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>123-456-7894</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>Silicon Valley, Zone 4</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>Extract B2B lead information for the tech sector in region 4.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>LEAD_GENERATION</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>FRESHER</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Tech Innovators 5 LLC</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://innovators5.io</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Jane Smith 5</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>CTO</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>jsmith5@innovators.io</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>https://linkedin.com/company/innovators5</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>123-456-7895</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>Silicon Valley, Zone 5</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>Extract B2B lead information for the tech sector in region 5.</t>
+          <t>tedt@atfco.com</t>
         </is>
       </c>
     </row>

</xml_diff>